<commit_message>
added logger winston and negative loigin scenarios
</commit_message>
<xml_diff>
--- a/test-data/Team01_The_Async_Actors_Test_Data.xlsx
+++ b/test-data/Team01_The_Async_Actors_Test_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maya/Documents/Maya Numpy Ninja/NUMPY PLAYWRIGHT/Team01_The_Async_Actors/test-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E77C3C58-B79E-DA47-9029-609BE329C832}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECF4DF1F-E824-1841-BBEB-0EC644BC4B29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16920" xr2:uid="{E7E101E1-228D-6542-9EA4-C401DB0741D4}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="21">
   <si>
     <t>Scenario</t>
   </si>
@@ -94,6 +94,15 @@
   </si>
   <si>
     <t>invalid_username</t>
+  </si>
+  <si>
+    <t>empty_password</t>
+  </si>
+  <si>
+    <t>Missing required field</t>
+  </si>
+  <si>
+    <t>empty_login</t>
   </si>
 </sst>
 </file>
@@ -465,7 +474,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0550789F-3113-2A45-80A7-74653352CE00}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.33203125" bestFit="1" customWidth="1"/>
@@ -512,6 +521,28 @@
       </c>
       <c r="D3" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
more scenarios in accounts
</commit_message>
<xml_diff>
--- a/test-data/Team01_The_Async_Actors_Test_Data.xlsx
+++ b/test-data/Team01_The_Async_Actors_Test_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maya/Documents/Maya Numpy Ninja/NUMPY PLAYWRIGHT/Team01_The_Async_Actors/test-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECF4DF1F-E824-1841-BBEB-0EC644BC4B29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE9F2CD4-5381-5D4E-A7E7-3D1700833905}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16920" xr2:uid="{E7E101E1-228D-6542-9EA4-C401DB0741D4}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16920" activeTab="1" xr2:uid="{E7E101E1-228D-6542-9EA4-C401DB0741D4}"/>
   </bookViews>
   <sheets>
     <sheet name="login" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
   <si>
     <t>Scenario</t>
   </si>
@@ -60,27 +60,12 @@
     <t>invalid_user</t>
   </si>
   <si>
-    <t>AccountName</t>
-  </si>
-  <si>
     <t>Phone</t>
   </si>
   <si>
     <t>Website</t>
   </si>
   <si>
-    <t>create_valid_account</t>
-  </si>
-  <si>
-    <t>Test Account 001</t>
-  </si>
-  <si>
-    <t>https://test1.com</t>
-  </si>
-  <si>
-    <t>success</t>
-  </si>
-  <si>
     <t>will</t>
   </si>
   <si>
@@ -103,6 +88,15 @@
   </si>
   <si>
     <t>empty_login</t>
+  </si>
+  <si>
+    <t>create_account_valid_name</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Numpy Test Account</t>
   </si>
 </sst>
 </file>
@@ -478,6 +472,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="37.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -497,7 +492,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s">
         <v>5</v>
@@ -506,43 +501,43 @@
         <v>4</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D5" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -556,9 +551,10 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="26.33203125" customWidth="1"/>
     <col min="4" max="4" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
@@ -566,13 +562,13 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" t="s">
         <v>6</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>7</v>
-      </c>
-      <c r="D1" t="s">
-        <v>8</v>
       </c>
       <c r="E1" t="s">
         <v>3</v>
@@ -580,19 +576,13 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2">
-        <v>15550100</v>
-      </c>
-      <c r="D2" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="E2" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added new feature for accoutn
</commit_message>
<xml_diff>
--- a/test-data/Team01_The_Async_Actors_Test_Data.xlsx
+++ b/test-data/Team01_The_Async_Actors_Test_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maya/Documents/Maya Numpy Ninja/NUMPY PLAYWRIGHT/Team01_The_Async_Actors/test-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE9F2CD4-5381-5D4E-A7E7-3D1700833905}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E367A90-44FE-594A-A0CE-8B0294F68997}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16920" activeTab="1" xr2:uid="{E7E101E1-228D-6542-9EA4-C401DB0741D4}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="40">
   <si>
     <t>Scenario</t>
   </si>
@@ -97,6 +97,69 @@
   </si>
   <si>
     <t>Numpy Test Account</t>
+  </si>
+  <si>
+    <t>create_account_complete_overview</t>
+  </si>
+  <si>
+    <t>Numpy Complete Overview Account</t>
+  </si>
+  <si>
+    <t>https://example.com</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>accounts@example.com</t>
+  </si>
+  <si>
+    <t>123 Billing Street</t>
+  </si>
+  <si>
+    <t>BillingStreet</t>
+  </si>
+  <si>
+    <t>BillingPostalCode</t>
+  </si>
+  <si>
+    <t>BillingCity</t>
+  </si>
+  <si>
+    <t>Boston</t>
+  </si>
+  <si>
+    <t>BillingState</t>
+  </si>
+  <si>
+    <t>Massachusetts</t>
+  </si>
+  <si>
+    <t>BillingCountry</t>
+  </si>
+  <si>
+    <t>USA</t>
+  </si>
+  <si>
+    <t>ShippingStreet</t>
+  </si>
+  <si>
+    <t>456 Shipping Avenue</t>
+  </si>
+  <si>
+    <t>ShippingPostalCode</t>
+  </si>
+  <si>
+    <t>ShippingCity</t>
+  </si>
+  <si>
+    <t>New York</t>
+  </si>
+  <si>
+    <t>ShippingState</t>
+  </si>
+  <si>
+    <t>ShippingCountry</t>
   </si>
 </sst>
 </file>
@@ -547,17 +610,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C58E1D24-B2F8-D748-9ED4-499650D2E4FA}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:R3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="26.33203125" customWidth="1"/>
     <col min="4" max="4" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -571,18 +637,101 @@
         <v>7</v>
       </c>
       <c r="E1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G1" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" t="s">
+        <v>29</v>
+      </c>
+      <c r="J1" t="s">
+        <v>31</v>
+      </c>
+      <c r="K1" t="s">
+        <v>33</v>
+      </c>
+      <c r="L1" t="s">
+        <v>35</v>
+      </c>
+      <c r="M1" t="s">
+        <v>36</v>
+      </c>
+      <c r="N1" t="s">
+        <v>38</v>
+      </c>
+      <c r="O1" t="s">
+        <v>39</v>
+      </c>
+      <c r="R1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
       <c r="B2" t="s">
         <v>18</v>
       </c>
-      <c r="E2" t="s">
+      <c r="R2" t="s">
         <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3">
+        <v>6175550100</v>
+      </c>
+      <c r="D3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G3">
+        <v>2108</v>
+      </c>
+      <c r="H3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I3" t="s">
+        <v>30</v>
+      </c>
+      <c r="J3" t="s">
+        <v>32</v>
+      </c>
+      <c r="K3" t="s">
+        <v>34</v>
+      </c>
+      <c r="L3">
+        <v>10001</v>
+      </c>
+      <c r="M3" t="s">
+        <v>37</v>
+      </c>
+      <c r="N3" t="s">
+        <v>37</v>
+      </c>
+      <c r="O3" t="s">
+        <v>32</v>
+      </c>
+      <c r="R3" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
code cleanup for step def
</commit_message>
<xml_diff>
--- a/test-data/Team01_The_Async_Actors_Test_Data.xlsx
+++ b/test-data/Team01_The_Async_Actors_Test_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maya/Documents/Maya Numpy Ninja/NUMPY PLAYWRIGHT/Team01_The_Async_Actors/test-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E06ADF75-D229-7841-8E05-4427F4CD1E5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DABF71ED-FEA3-DA49-B661-A026C885D187}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16920" activeTab="1" xr2:uid="{E7E101E1-228D-6542-9EA4-C401DB0741D4}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="65">
   <si>
     <t>Scenario</t>
   </si>
@@ -229,6 +229,12 @@
   </si>
   <si>
     <t>Numpy Account Partial Search Test</t>
+  </si>
+  <si>
+    <t>Numpy Account Partial</t>
+  </si>
+  <si>
+    <t>SearchText</t>
   </si>
 </sst>
 </file>
@@ -686,20 +692,21 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C58E1D24-B2F8-D748-9ED4-499650D2E4FA}">
-  <dimension ref="A1:R11"/>
+  <dimension ref="A1:S11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="30.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.33203125" customWidth="1"/>
-    <col min="4" max="4" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.5" customWidth="1"/>
+    <col min="4" max="4" width="26.33203125" customWidth="1"/>
+    <col min="5" max="5" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="13.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -707,203 +714,209 @@
         <v>17</v>
       </c>
       <c r="C1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D1" t="s">
         <v>6</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>7</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>22</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>25</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>26</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>27</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>29</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>31</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>33</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>35</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>36</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>38</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>39</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
       <c r="B2" t="s">
         <v>18</v>
       </c>
-      <c r="R2" t="s">
+      <c r="S2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>19</v>
       </c>
       <c r="B3" t="s">
         <v>20</v>
       </c>
-      <c r="C3">
+      <c r="D3">
         <v>6175550100</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>21</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>23</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>24</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>2108</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>28</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>30</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>32</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>34</v>
       </c>
-      <c r="L3">
+      <c r="M3">
         <v>10001</v>
-      </c>
-      <c r="M3" t="s">
-        <v>37</v>
       </c>
       <c r="N3" t="s">
         <v>37</v>
       </c>
       <c r="O3" t="s">
+        <v>37</v>
+      </c>
+      <c r="P3" t="s">
         <v>32</v>
       </c>
-      <c r="R3" t="s">
+      <c r="S3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>40</v>
       </c>
       <c r="B4" t="s">
         <v>41</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>42</v>
       </c>
-      <c r="R4" t="s">
+      <c r="S4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>43</v>
       </c>
       <c r="B5" t="s">
         <v>44</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>45</v>
       </c>
-      <c r="R5" t="s">
+      <c r="S5" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>47</v>
       </c>
       <c r="B6" t="s">
         <v>48</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>49</v>
       </c>
-      <c r="R6" t="s">
+      <c r="S6" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>51</v>
       </c>
       <c r="B7" t="s">
         <v>61</v>
       </c>
-      <c r="R7" t="s">
+      <c r="S7" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>52</v>
       </c>
       <c r="B8" t="s">
         <v>62</v>
       </c>
-      <c r="R8" t="s">
+      <c r="C8" t="s">
+        <v>63</v>
+      </c>
+      <c r="S8" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>53</v>
       </c>
       <c r="B9" t="s">
         <v>54</v>
       </c>
-      <c r="R9" t="s">
+      <c r="S9" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>56</v>
       </c>
       <c r="B10" t="s">
         <v>58</v>
       </c>
-      <c r="R10" t="s">
+      <c r="S10" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="17" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:19" ht="17" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>57</v>
       </c>
       <c r="B11" t="s">
         <v>59</v>
       </c>
-      <c r="R11" s="1" t="s">
+      <c r="S11" s="1" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added new featires for oppurtunites
</commit_message>
<xml_diff>
--- a/test-data/Team01_The_Async_Actors_Test_Data.xlsx
+++ b/test-data/Team01_The_Async_Actors_Test_Data.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maya/Documents/Maya Numpy Ninja/NUMPY PLAYWRIGHT/Team01_The_Async_Actors/test-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79EDC3D9-B434-8744-9090-DEEF121E4C96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5A98429-2451-B248-9F92-659C395A626D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16920" activeTab="1" xr2:uid="{E7E101E1-228D-6542-9EA4-C401DB0741D4}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16920" activeTab="2" xr2:uid="{E7E101E1-228D-6542-9EA4-C401DB0741D4}"/>
   </bookViews>
   <sheets>
     <sheet name="login" sheetId="1" r:id="rId1"/>
     <sheet name="Accounts" sheetId="2" r:id="rId2"/>
+    <sheet name="opputinuites" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="86">
   <si>
     <t>Scenario</t>
   </si>
@@ -268,6 +269,36 @@
   </si>
   <si>
     <t>https://changed.example.com</t>
+  </si>
+  <si>
+    <t>OpportunityName</t>
+  </si>
+  <si>
+    <t>AccountName</t>
+  </si>
+  <si>
+    <t>OpportunityAmount</t>
+  </si>
+  <si>
+    <t>create_opportunity_valid_mandatory</t>
+  </si>
+  <si>
+    <t>Numpy Test Opportunity</t>
+  </si>
+  <si>
+    <t>Numpy Test Oppurtunity Account</t>
+  </si>
+  <si>
+    <t>SalesStage</t>
+  </si>
+  <si>
+    <t>ExpectedCloseDate</t>
+  </si>
+  <si>
+    <t>Negotiation/Review</t>
+  </si>
+  <si>
+    <t>'2027-03-15</t>
   </si>
 </sst>
 </file>
@@ -309,9 +340,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1014,4 +1046,61 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC6EEF89-D845-DA44-8C07-7269BB5340C5}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="31.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="23.5" customWidth="1"/>
+    <col min="5" max="5" width="17.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D2">
+        <v>5000</v>
+      </c>
+      <c r="E2" t="s">
+        <v>84</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
added more scenarios for opputunity
</commit_message>
<xml_diff>
--- a/test-data/Team01_The_Async_Actors_Test_Data.xlsx
+++ b/test-data/Team01_The_Async_Actors_Test_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maya/Documents/Maya Numpy Ninja/NUMPY PLAYWRIGHT/Team01_The_Async_Actors/test-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AB3B27C-9833-F449-AA14-CB269B0D10A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF68D298-D48E-384E-B935-A4F1BDFB931F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16920" activeTab="2" xr2:uid="{E7E101E1-228D-6542-9EA4-C401DB0741D4}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="161">
   <si>
     <t>Scenario</t>
   </si>
@@ -329,6 +329,201 @@
   </si>
   <si>
     <t>$</t>
+  </si>
+  <si>
+    <t>create_opportunity_existing_business</t>
+  </si>
+  <si>
+    <t>Numpy Existing Business Opportunity</t>
+  </si>
+  <si>
+    <t>Numpy Existing Business Account</t>
+  </si>
+  <si>
+    <t>OpportunityType</t>
+  </si>
+  <si>
+    <t>Existing Business</t>
+  </si>
+  <si>
+    <t>create_opportunity_new_business</t>
+  </si>
+  <si>
+    <t>Numpy New Business Opportunity</t>
+  </si>
+  <si>
+    <t>Numpy New Business Account</t>
+  </si>
+  <si>
+    <t>New Business</t>
+  </si>
+  <si>
+    <t>create_opportunity_lead_source_cold_call</t>
+  </si>
+  <si>
+    <t>create_opportunity_lead_source_existing_customer</t>
+  </si>
+  <si>
+    <t>create_opportunity_lead_source_self_generated</t>
+  </si>
+  <si>
+    <t>create_opportunity_lead_source_employee</t>
+  </si>
+  <si>
+    <t>create_opportunity_lead_source_partner</t>
+  </si>
+  <si>
+    <t>create_opportunity_lead_source_public_relations</t>
+  </si>
+  <si>
+    <t>create_opportunity_lead_source_direct_mail</t>
+  </si>
+  <si>
+    <t>create_opportunity_lead_source_conference</t>
+  </si>
+  <si>
+    <t>create_opportunity_lead_source_trade_show</t>
+  </si>
+  <si>
+    <t>create_opportunity_lead_source_web_site</t>
+  </si>
+  <si>
+    <t>create_opportunity_lead_source_word_of_mouth</t>
+  </si>
+  <si>
+    <t>create_opportunity_lead_source_email</t>
+  </si>
+  <si>
+    <t>create_opportunity_lead_source_campaign</t>
+  </si>
+  <si>
+    <t>create_opportunity_lead_source_other</t>
+  </si>
+  <si>
+    <t>Numpy Cold Call Opportunity</t>
+  </si>
+  <si>
+    <t>Numpy Existing Customer Opportunity</t>
+  </si>
+  <si>
+    <t>Numpy Self Generated Opportunity</t>
+  </si>
+  <si>
+    <t>Numpy Employee Opportunity</t>
+  </si>
+  <si>
+    <t>Numpy Partner Opportunity</t>
+  </si>
+  <si>
+    <t>Numpy Public Relations Opportunity</t>
+  </si>
+  <si>
+    <t>Numpy Direct Mail Opportunity</t>
+  </si>
+  <si>
+    <t>Numpy Conference Opportunity</t>
+  </si>
+  <si>
+    <t>Numpy Trade Show Opportunity</t>
+  </si>
+  <si>
+    <t>Numpy Web Site Opportunity</t>
+  </si>
+  <si>
+    <t>Numpy Word of Mouth Opportunity</t>
+  </si>
+  <si>
+    <t>Numpy Email Opportunity</t>
+  </si>
+  <si>
+    <t>Numpy Campaign Opportunity</t>
+  </si>
+  <si>
+    <t>Numpy Other Opportunity</t>
+  </si>
+  <si>
+    <t>Numpy Cold Call Account</t>
+  </si>
+  <si>
+    <t>Numpy Existing Customer Account</t>
+  </si>
+  <si>
+    <t>Numpy Self Generated Account</t>
+  </si>
+  <si>
+    <t>Numpy Employee Account</t>
+  </si>
+  <si>
+    <t>Numpy Partner Account</t>
+  </si>
+  <si>
+    <t>Numpy Public Relations Account</t>
+  </si>
+  <si>
+    <t>Numpy Direct Mail Account</t>
+  </si>
+  <si>
+    <t>Numpy Conference Account</t>
+  </si>
+  <si>
+    <t>Numpy Trade Show Account</t>
+  </si>
+  <si>
+    <t>Numpy Web Site Account</t>
+  </si>
+  <si>
+    <t>Numpy Word of Mouth Account</t>
+  </si>
+  <si>
+    <t>Numpy Email Account</t>
+  </si>
+  <si>
+    <t>Numpy Campaign Account</t>
+  </si>
+  <si>
+    <t>Numpy Other Account</t>
+  </si>
+  <si>
+    <t>LeadSource</t>
+  </si>
+  <si>
+    <t>Cold Call</t>
+  </si>
+  <si>
+    <t>Existing Customer</t>
+  </si>
+  <si>
+    <t>Self Generated</t>
+  </si>
+  <si>
+    <t>Employee</t>
+  </si>
+  <si>
+    <t>Partner</t>
+  </si>
+  <si>
+    <t>Public Relations</t>
+  </si>
+  <si>
+    <t>Direct Mail</t>
+  </si>
+  <si>
+    <t>Conference</t>
+  </si>
+  <si>
+    <t>Trade Show</t>
+  </si>
+  <si>
+    <t>Web Site</t>
+  </si>
+  <si>
+    <t>Word of mouth</t>
+  </si>
+  <si>
+    <t>Campaign</t>
+  </si>
+  <si>
+    <t>Other</t>
   </si>
 </sst>
 </file>
@@ -1080,19 +1275,21 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC6EEF89-D845-DA44-8C07-7269BB5340C5}">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="31.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="1" max="1" width="43.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="23.5" customWidth="1"/>
     <col min="5" max="5" width="17.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17.5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1117,8 +1314,14 @@
       <c r="H1" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I1" t="s">
+        <v>99</v>
+      </c>
+      <c r="J1" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>79</v>
       </c>
@@ -1138,7 +1341,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>85</v>
       </c>
@@ -1158,7 +1361,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>89</v>
       </c>
@@ -1182,6 +1385,374 @@
       </c>
       <c r="H4" t="s">
         <v>95</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>96</v>
+      </c>
+      <c r="B5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C5" t="s">
+        <v>98</v>
+      </c>
+      <c r="D5">
+        <v>7500.5</v>
+      </c>
+      <c r="E5" t="s">
+        <v>84</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="I5" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>101</v>
+      </c>
+      <c r="B6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6" t="s">
+        <v>103</v>
+      </c>
+      <c r="D6">
+        <v>8500.5</v>
+      </c>
+      <c r="E6" t="s">
+        <v>84</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="I6" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>105</v>
+      </c>
+      <c r="B7" t="s">
+        <v>119</v>
+      </c>
+      <c r="C7" t="s">
+        <v>133</v>
+      </c>
+      <c r="D7">
+        <v>7500.5</v>
+      </c>
+      <c r="E7" t="s">
+        <v>84</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="J7" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>106</v>
+      </c>
+      <c r="B8" t="s">
+        <v>120</v>
+      </c>
+      <c r="C8" t="s">
+        <v>134</v>
+      </c>
+      <c r="D8">
+        <v>7500.5</v>
+      </c>
+      <c r="E8" t="s">
+        <v>84</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="J8" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>107</v>
+      </c>
+      <c r="B9" t="s">
+        <v>121</v>
+      </c>
+      <c r="C9" t="s">
+        <v>135</v>
+      </c>
+      <c r="D9">
+        <v>7500.5</v>
+      </c>
+      <c r="E9" t="s">
+        <v>84</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="J9" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>108</v>
+      </c>
+      <c r="B10" t="s">
+        <v>122</v>
+      </c>
+      <c r="C10" t="s">
+        <v>136</v>
+      </c>
+      <c r="D10">
+        <v>7500.5</v>
+      </c>
+      <c r="E10" t="s">
+        <v>84</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="J10" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>109</v>
+      </c>
+      <c r="B11" t="s">
+        <v>123</v>
+      </c>
+      <c r="C11" t="s">
+        <v>137</v>
+      </c>
+      <c r="D11">
+        <v>7500.5</v>
+      </c>
+      <c r="E11" t="s">
+        <v>84</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="J11" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>110</v>
+      </c>
+      <c r="B12" t="s">
+        <v>124</v>
+      </c>
+      <c r="C12" t="s">
+        <v>138</v>
+      </c>
+      <c r="D12">
+        <v>7500.5</v>
+      </c>
+      <c r="E12" t="s">
+        <v>84</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="J12" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>111</v>
+      </c>
+      <c r="B13" t="s">
+        <v>125</v>
+      </c>
+      <c r="C13" t="s">
+        <v>139</v>
+      </c>
+      <c r="D13">
+        <v>7500.5</v>
+      </c>
+      <c r="E13" t="s">
+        <v>84</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="J13" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>112</v>
+      </c>
+      <c r="B14" t="s">
+        <v>126</v>
+      </c>
+      <c r="C14" t="s">
+        <v>140</v>
+      </c>
+      <c r="D14">
+        <v>7500.5</v>
+      </c>
+      <c r="E14" t="s">
+        <v>84</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="J14" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>113</v>
+      </c>
+      <c r="B15" t="s">
+        <v>127</v>
+      </c>
+      <c r="C15" t="s">
+        <v>141</v>
+      </c>
+      <c r="D15">
+        <v>7500.5</v>
+      </c>
+      <c r="E15" t="s">
+        <v>84</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="J15" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>114</v>
+      </c>
+      <c r="B16" t="s">
+        <v>128</v>
+      </c>
+      <c r="C16" t="s">
+        <v>142</v>
+      </c>
+      <c r="D16">
+        <v>7500.5</v>
+      </c>
+      <c r="E16" t="s">
+        <v>84</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="J16" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>115</v>
+      </c>
+      <c r="B17" t="s">
+        <v>129</v>
+      </c>
+      <c r="C17" t="s">
+        <v>143</v>
+      </c>
+      <c r="D17">
+        <v>7500.5</v>
+      </c>
+      <c r="E17" t="s">
+        <v>84</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="J17" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>116</v>
+      </c>
+      <c r="B18" t="s">
+        <v>130</v>
+      </c>
+      <c r="C18" t="s">
+        <v>144</v>
+      </c>
+      <c r="D18">
+        <v>7500.5</v>
+      </c>
+      <c r="E18" t="s">
+        <v>84</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="J18" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>117</v>
+      </c>
+      <c r="B19" t="s">
+        <v>131</v>
+      </c>
+      <c r="C19" t="s">
+        <v>145</v>
+      </c>
+      <c r="D19">
+        <v>7500.5</v>
+      </c>
+      <c r="E19" t="s">
+        <v>84</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="J19" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>118</v>
+      </c>
+      <c r="B20" t="s">
+        <v>132</v>
+      </c>
+      <c r="C20" t="s">
+        <v>146</v>
+      </c>
+      <c r="D20">
+        <v>7500.5</v>
+      </c>
+      <c r="E20" t="s">
+        <v>84</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="J20" t="s">
+        <v>160</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added scenario for oppurtinuiyy
</commit_message>
<xml_diff>
--- a/test-data/Team01_The_Async_Actors_Test_Data.xlsx
+++ b/test-data/Team01_The_Async_Actors_Test_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maya/Documents/Maya Numpy Ninja/NUMPY PLAYWRIGHT/Team01_The_Async_Actors/test-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF68D298-D48E-384E-B935-A4F1BDFB931F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5908C3E-C9FA-2444-A4CE-D6A5E6884803}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16920" activeTab="2" xr2:uid="{E7E101E1-228D-6542-9EA4-C401DB0741D4}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="166">
   <si>
     <t>Scenario</t>
   </si>
@@ -524,6 +524,21 @@
   </si>
   <si>
     <t>Other</t>
+  </si>
+  <si>
+    <t>create_opportunity_with_description</t>
+  </si>
+  <si>
+    <t>Numpy Description Opportunity</t>
+  </si>
+  <si>
+    <t>Numpy Description Account</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Opportunity created to verify that the entered description is saved</t>
   </si>
 </sst>
 </file>
@@ -1275,7 +1290,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC6EEF89-D845-DA44-8C07-7269BB5340C5}">
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="43.83203125" bestFit="1" customWidth="1"/>
@@ -1289,7 +1304,7 @@
     <col min="9" max="9" width="14.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1320,8 +1335,11 @@
       <c r="J1" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K1" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>79</v>
       </c>
@@ -1341,7 +1359,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>85</v>
       </c>
@@ -1361,7 +1379,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>89</v>
       </c>
@@ -1387,7 +1405,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>96</v>
       </c>
@@ -1410,7 +1428,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>101</v>
       </c>
@@ -1433,7 +1451,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>105</v>
       </c>
@@ -1456,7 +1474,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>106</v>
       </c>
@@ -1479,7 +1497,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>107</v>
       </c>
@@ -1502,7 +1520,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>108</v>
       </c>
@@ -1525,7 +1543,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>109</v>
       </c>
@@ -1548,7 +1566,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>110</v>
       </c>
@@ -1571,7 +1589,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>111</v>
       </c>
@@ -1594,7 +1612,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>112</v>
       </c>
@@ -1617,7 +1635,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>113</v>
       </c>
@@ -1640,7 +1658,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>114</v>
       </c>
@@ -1663,7 +1681,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>115</v>
       </c>
@@ -1686,7 +1704,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>116</v>
       </c>
@@ -1709,7 +1727,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>117</v>
       </c>
@@ -1732,7 +1750,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>118</v>
       </c>
@@ -1753,6 +1771,29 @@
       </c>
       <c r="J20" t="s">
         <v>160</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>161</v>
+      </c>
+      <c r="B21" t="s">
+        <v>162</v>
+      </c>
+      <c r="C21" t="s">
+        <v>163</v>
+      </c>
+      <c r="D21">
+        <v>7500.5</v>
+      </c>
+      <c r="E21" t="s">
+        <v>84</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="K21" t="s">
+        <v>165</v>
       </c>
     </row>
   </sheetData>

</xml_diff>